<commit_message>
🔄 Index Monitor Update - 2026-07-23 03:15:08 UTC
Detected 6 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -513,42 +513,42 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>National Storage Affiliates Trust</t>
+          <t>Taylor Morrison Home</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>0001618563</t>
+          <t>0001562476</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>NSA</t>
+          <t>TMHC</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Molina Healthcare</t>
+          <t>Krystal Biotech</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>0001179929</t>
+          <t>0001711279</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>MOH</t>
+          <t>KRYS</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -565,22 +565,22 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 400</t>
+          <t>S&amp;P 600</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Taylor Morrison Home</t>
+          <t>Krystal Biotech</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>0001562476</t>
+          <t>0001711279</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>TMHC</t>
+          <t>KRYS</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -590,17 +590,17 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Krystal Biotech</t>
+          <t>Tutor Perini Corp</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>0001711279</t>
+          <t>0000077543</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>KRYS</t>
+          <t>TPC</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -627,42 +627,42 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Molina Healthcare</t>
+          <t>Avanos Medical</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>0001179929</t>
+          <t>0001606498</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>MOH</t>
+          <t>AVNS</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Construction Partners</t>
+          <t>V2X</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>0001718227</t>
+          <t>0001601548</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>ROAD</t>
+          <t>VVX</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -671,120 +671,6 @@
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Krystal Biotech</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>0001711279</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>KRYS</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Tutor Perini Corp</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>0000077543</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>TPC</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Avanos Medical</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>0001606498</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>AVNS</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>V2X</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>0001601548</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>VVX</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>10-Q filed in 2026</t>
         </is>
@@ -801,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -858,22 +744,22 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Molina Healthcare</t>
+          <t>Krystal Biotech</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>0001179929</t>
+          <t>0001711279</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>MOH</t>
+          <t>KRYS</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -895,22 +781,22 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>National Storage Affiliates Trust</t>
+          <t>Taylor Morrison Home</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>0001618563</t>
+          <t>0001562476</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>NSA</t>
+          <t>TMHC</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -927,7 +813,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 400</t>
+          <t>S&amp;P 600</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -952,7 +838,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Added</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -964,22 +850,22 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 400</t>
+          <t>S&amp;P 600</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Taylor Morrison Home</t>
+          <t>Tutor Perini Corp</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>0001562476</t>
+          <t>0000077543</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>TMHC</t>
+          <t>TPC</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -989,12 +875,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>DEFM14A filed in 2026</t>
+          <t>10-Q filed in 2026</t>
         </is>
       </c>
     </row>
@@ -1006,32 +892,32 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Construction Partners</t>
+          <t>Avanos Medical</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>0001718227</t>
+          <t>0001606498</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>ROAD</t>
+          <t>AVNS</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Added</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>10-Q filed in 2026</t>
+          <t>DEFA14A filed in 2026</t>
         </is>
       </c>
     </row>
@@ -1043,178 +929,30 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Molina Healthcare</t>
+          <t>V2X</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>0001179929</t>
+          <t>0001601548</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>MOH</t>
+          <t>VVX</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Krystal Biotech</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>0001711279</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>KRYS</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Tutor Perini Corp</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>0000077543</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>TPC</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Avanos Medical</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>0001606498</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>AVNS</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>DEFA14A filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>V2X</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>0001601548</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>VVX</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>10-Q filed in 2026</t>
         </is>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-07-25 02:54:00 UTC
Detected 2 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -508,47 +508,47 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 400</t>
+          <t>S&amp;P 600</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Taylor Morrison Home</t>
+          <t>Avanos Medical</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>0001562476</t>
+          <t>0001606498</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TMHC</t>
+          <t>AVNS</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Krystal Biotech</t>
+          <t>V2X</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>0001711279</t>
+          <t>0001601548</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>KRYS</t>
+          <t>VVX</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -557,120 +557,6 @@
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Krystal Biotech</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>0001711279</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>KRYS</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Tutor Perini Corp</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>0000077543</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>TPC</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Avanos Medical</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>0001606498</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>AVNS</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>V2X</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>0001601548</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>VVX</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>10-Q filed in 2026</t>
         </is>
@@ -687,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -739,220 +625,72 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 400</t>
+          <t>S&amp;P 600</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Krystal Biotech</t>
+          <t>Avanos Medical</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>0001711279</t>
+          <t>0001606498</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>KRYS</t>
+          <t>AVNS</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Added</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>10-Q filed in 2026</t>
+          <t>DEFA14A filed in 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 400</t>
+          <t>S&amp;P 600</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Taylor Morrison Home</t>
+          <t>V2X</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>0001562476</t>
+          <t>0001601548</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>TMHC</t>
+          <t>VVX</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>DEFM14A filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Krystal Biotech</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>0001711279</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>KRYS</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Tutor Perini Corp</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>0000077543</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>TPC</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Avanos Medical</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>0001606498</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>AVNS</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>DEFA14A filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>V2X</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>0001601548</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>VVX</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>10-Q filed in 2026</t>
         </is>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-07-25 19:12:55 UTC
Detected 0 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -34,7 +34,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -508,57 +510,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Avanos Medical</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0001606498</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>AVNS</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>V2X</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>0001601548</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>VVX</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
+          <t>(no going-forward changes found in this run)</t>
         </is>
       </c>
     </row>
@@ -573,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -625,74 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Avanos Medical</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0001606498</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>AVNS</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>DEFA14A filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>V2X</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>0001601548</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>VVX</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
+          <t>(no going-forward changes found in this run)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-07-26 03:19:24 UTC
Detected 2 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -34,9 +34,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -510,7 +508,57 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(no going-forward changes found in this run)</t>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Avanos Medical</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0001606498</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>AVNS</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>V2X</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>0001601548</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>VVX</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
         </is>
       </c>
     </row>
@@ -525,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -577,7 +625,74 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(no going-forward changes found in this run)</t>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Avanos Medical</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0001606498</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>AVNS</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>DEFA14A filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>V2X</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>0001601548</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>VVX</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-07-26 08:32:41 UTC
Detected 0 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -34,7 +34,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -508,57 +510,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Avanos Medical</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0001606498</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>AVNS</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>V2X</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>0001601548</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>VVX</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
+          <t>(no going-forward changes found in this run)</t>
         </is>
       </c>
     </row>
@@ -573,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -625,74 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Avanos Medical</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0001606498</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>AVNS</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>DEFA14A filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>V2X</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>0001601548</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>VVX</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
+          <t>(no going-forward changes found in this run)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-07-26 13:36:35 UTC
Detected 2 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -34,9 +34,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -510,7 +508,57 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(no going-forward changes found in this run)</t>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Avanos Medical</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0001606498</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>AVNS</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>V2X</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>0001601548</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>VVX</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
         </is>
       </c>
     </row>
@@ -525,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -577,7 +625,74 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(no going-forward changes found in this run)</t>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Avanos Medical</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0001606498</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>AVNS</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>DEFA14A filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>V2X</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>0001601548</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>VVX</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-07-28 02:46:07 UTC
Detected 0 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -34,7 +34,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -508,57 +510,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Avanos Medical</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0001606498</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>AVNS</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>V2X</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>0001601548</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>VVX</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
+          <t>(no going-forward changes found in this run)</t>
         </is>
       </c>
     </row>
@@ -573,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -625,74 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Avanos Medical</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0001606498</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>AVNS</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>DEFA14A filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>V2X</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>0001601548</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>VVX</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
+          <t>(no going-forward changes found in this run)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-07-30 02:38:03 UTC
Detected 2 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -34,9 +34,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -510,7 +508,57 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(no going-forward changes found in this run)</t>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Two Harbors Investment</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0001465740</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>TWO</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Five9</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>0001288847</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>FIVN</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
         </is>
       </c>
     </row>
@@ -525,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -577,7 +625,74 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(no going-forward changes found in this run)</t>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Five9</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0001288847</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>FIVN</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Two Harbors Investment</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>0001465740</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>TWO</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-08-01 03:17:21 UTC
Detected 6 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -508,57 +508,171 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Electronic Arts</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0000712515</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Ferguson Enterprises</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>0002011641</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>FERG</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
           <t>S&amp;P 600</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Two Harbors Investment</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>0001465740</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>TWO</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Five9</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>0001288847</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>FIVN</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Same effective date</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>10-Q filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Hertz Global Holdings</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>0001657853</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>HTZ</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>ADI Global Distribution</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>0002105139</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>ADIG</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Different effective dates — paired for reference only</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>New cik Yet not filed 10-K or 10-Q</t>
         </is>
       </c>
     </row>
@@ -573,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -625,72 +739,220 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
+          <t>S&amp;P 500</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Electronic Arts</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>0001288847</t>
+          <t>0000712515</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>FIVN</t>
+          <t>EA</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Added</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>10-Q filed in 2026</t>
+          <t>10-K/A filed in 2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Ferguson Enterprises</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>0002011641</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>FERG</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
           <t>S&amp;P 600</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Five9</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>0001288847</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>FIVN</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Two Harbors Investment</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>0001465740</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>TWO</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Removed</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>ADI Global Distribution</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>0002105139</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ADIG</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>New cik Yet not filed 10-K or 10-Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Hertz Global Holdings</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>0001657853</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>HTZ</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>10-Q filed in 2026</t>
         </is>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-08-04 02:48:50 UTC
Detected 4 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -570,107 +570,50 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Two Harbors Investment</t>
+          <t>Hertz Global Holdings</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>0001465740</t>
+          <t>0001657853</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>TWO</t>
+          <t>HTZ</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>ADI Global Distribution</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>0001288847</t>
+          <t>0002105139</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>FIVN</t>
+          <t>ADIG</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Same effective date</t>
+          <t>Different effective dates — paired for reference only</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Hertz Global Holdings</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>0001657853</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>HTZ</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>ADI Global Distribution</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>0002105139</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>ADIG</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-04</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Different effective dates — paired for reference only</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>New cik Yet not filed 10-K or 10-Q</t>
         </is>
@@ -687,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -769,7 +712,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>10-K/A filed in 2026</t>
+          <t>10-Q filed in 2026</t>
         </is>
       </c>
     </row>
@@ -818,22 +761,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>ADI Global Distribution</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>0001288847</t>
+          <t>0002105139</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>FIVN</t>
+          <t>ADIG</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -843,7 +786,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>10-Q filed in 2026</t>
+          <t>New cik Yet not filed 10-K or 10-Q</t>
         </is>
       </c>
     </row>
@@ -855,22 +798,22 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Two Harbors Investment</t>
+          <t>Hertz Global Holdings</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>0001465740</t>
+          <t>0001657853</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>TWO</t>
+          <t>HTZ</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -879,80 +822,6 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>ADI Global Distribution</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>0002105139</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>ADIG</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-04</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>New cik Yet not filed 10-K or 10-Q</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Hertz Global Holdings</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>0001657853</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>HTZ</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>10-Q filed in 2026</t>
         </is>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-08-05 02:46:14 UTC
Detected 3 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -588,36 +588,16 @@
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>ADI Global Distribution</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>0002105139</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>ADIG</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-04</t>
-        </is>
-      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Different effective dates — paired for reference only</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>New cik Yet not filed 10-K or 10-Q</t>
-        </is>
-      </c>
+          <t>Removed, no matching addition found</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -630,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -761,67 +741,30 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ADI Global Distribution</t>
+          <t>Hertz Global Holdings</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>0002105139</t>
+          <t>0001657853</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>ADIG</t>
+          <t>HTZ</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Added</t>
+          <t>Removed</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>New cik Yet not filed 10-K or 10-Q</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Hertz Global Holdings</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>0001657853</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>HTZ</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>10-Q filed in 2026</t>
         </is>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-08-06 02:48:55 UTC
Detected 0 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -34,7 +34,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -432,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -508,96 +510,9 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 500</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Electronic Arts</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0000712515</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Ferguson Enterprises</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>0002011641</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>FERG</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Hertz Global Holdings</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>0001657853</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>HTZ</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Removed, no matching addition found</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr"/>
+          <t>(no going-forward changes found in this run)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -610,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -662,111 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 500</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Electronic Arts</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0000712515</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 500</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Ferguson Enterprises</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>0002011641</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>FERG</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Hertz Global Holdings</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>0001657853</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>HTZ</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
+          <t>(no going-forward changes found in this run)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-08-14 02:10:10 UTC
Detected 4 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -34,9 +34,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -434,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -510,7 +508,114 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(no going-forward changes found in this run)</t>
+          <t>S&amp;P 400</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Webster Financial</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0000801337</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>WBS</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Sun Communities</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>0000912593</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>SUI</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>AvalonBay Communities</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>0000915912</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>AVB</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Reddit</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>0001713445</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
         </is>
       </c>
     </row>
@@ -525,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -577,7 +682,148 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(no going-forward changes found in this run)</t>
+          <t>S&amp;P 400</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Sun Communities</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0000912593</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>SUI</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 400</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Webster Financial</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>0000801337</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>WBS</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>AvalonBay Communities</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>0000915912</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>AVB</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Reddit</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>0001713445</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-08-19 01:24:01 UTC
Detected 2 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -562,63 +562,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 500</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>AvalonBay Communities</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>0000915912</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>AVB</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Reddit</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>0001713445</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>RDDT</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -630,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -753,80 +696,6 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 500</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>AvalonBay Communities</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>0000915912</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>AVB</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 500</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Reddit</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>0001713445</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>RDDT</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-08-21 02:59:56 UTC
Detected 0 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -34,7 +34,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -508,57 +510,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 400</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Webster Financial</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0000801337</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>WBS</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Sun Communities</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>0000912593</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>SUI</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
+          <t>(no going-forward changes found in this run)</t>
         </is>
       </c>
     </row>
@@ -573,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -625,74 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 400</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Sun Communities</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0000912593</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>SUI</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 400</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Webster Financial</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>0000801337</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>WBS</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
+          <t>(no going-forward changes found in this run)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-08-27 04:29:08 UTC
Detected 2 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -34,9 +34,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -510,7 +508,57 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(no going-forward changes found in this run)</t>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Leggett &amp; Platt</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0000058492</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>LEG</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Tenable Holdings</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>0001660280</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
         </is>
       </c>
     </row>
@@ -525,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -577,7 +625,74 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(no going-forward changes found in this run)</t>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Leggett &amp; Platt</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0000058492</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>LEG</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Tenable Holdings</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>0001660280</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>TENB</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>10-Q filed in 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-09-01 03:45:18 UTC
Detected 0 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -34,7 +34,9 @@
     </font>
     <font>
       <name val="Arial"/>
-      <sz val="10"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -508,57 +510,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Leggett &amp; Platt</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0000058492</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>LEG</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Tenable Holdings</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>0001660280</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>TENB</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Same effective date</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
+          <t>(no going-forward changes found in this run)</t>
         </is>
       </c>
     </row>
@@ -573,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -625,74 +577,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Leggett &amp; Platt</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>0000058492</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>LEG</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>S&amp;P 600</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Tenable Holdings</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>0001660280</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>TENB</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>10-Q filed in 2026</t>
+          <t>(no going-forward changes found in this run)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔄 Index Monitor Update - 2026-09-07 05:13:29 UTC
Detected 21 going-forward index changes

Automated commit by GitHub Actions
</commit_message>
<xml_diff>
--- a/index_changes_going_forward.xlsx
+++ b/index_changes_going_forward.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Side by side" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Add remove version" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,9 +33,13 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="9"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -65,10 +68,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,20 +438,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -463,125 +466,1085 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Removed Cik</t>
+          <t>Removed Ticker</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Removed Ticker</t>
+          <t>Removed date</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Removed date</t>
+          <t>Added</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Added</t>
+          <t>Added Ticker</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Added CIK</t>
+          <t>Commencing date</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Added Ticker</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Commencing date</t>
+          <t>Reason</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Added latest filings</t>
+          <t>Refer Link</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(no going-forward changes found in this run)</t>
+          <t>S&amp;P 100</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Colgate-Palmolive</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Arista Networks</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 100</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Honeywell Aerospace</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>HONA</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Dell Technologies</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 100</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>NIKE</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Palo Alto Networks</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>PANW</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 100</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Simon Property Group</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>SPG</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 400</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Boston Beer</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>SAM</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>AGNC Investment</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>AGNC</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 400</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Capri Holdings</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>CPRI</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Brinker Intl</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>EAT</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 400</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Everpure</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Corcept Therapeutics</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>CORT</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 400</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Illumina</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>HubSpot</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>HUBS</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Builders FirstSource</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>BLDR</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Bloom Energy</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Molson Coors Beverage</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>TAP</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Everpure</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 500</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>The Trade Desk</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Illumina</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Amerisafe</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>AMSF</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>AXT</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>AXTI</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Brinker Intl</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>EAT</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Arcutis Biotherapeutics</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>ARQT</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Cogent Communications Holdings</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>CCOI</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>AtriCure</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>ATRC</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Corcept Therapeutics</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>CORT</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Boston Beer</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>SAM</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Franklin BSP Realty Trust</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>FBRT</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Builders FirstSource</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>BLDR</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Matthews Intl</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>MATW</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Capri Holdings</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>CPRI</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>N-able</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>NABL</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Delek US Holdings</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>NexPoint Residential Trust</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>NXRT</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Herc Holdings</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>HRI</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Shenandoah Telecommunications</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>SHEN</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Molson Coors Beverage</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>TAP</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>S&amp;P 600</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Verra Mobility</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>VRRM</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>The Trade Desk</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>TTD</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Same effective date</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Merger/Acquisition: News in Focus Browse News Releases All News Releases All Public Company English-only News Releases Overview Multimedia Gallery All Multimedia All Photos All Videos Multimedia Gallery Overview Trending Topics All Trending Topics Business &amp; Money Auto &amp; Transportation All Automo...</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.prnewswire.com/news-releases/bloom-energy-illumina-and-everpure-set-to-join-sp-500-others-to-join-sp-100-sp-midcap-400-and-sp-smallcap-600-302870517.html</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Indices</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Company name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Cik code</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Commencing date</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Latest Filing</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>(no going-forward changes found in this run)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId21"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>